<commit_message>
Add UART and echo program
</commit_message>
<xml_diff>
--- a/Instructions.xlsx
+++ b/Instructions.xlsx
@@ -1442,7 +1442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E57"/>
+  <dimension ref="A2:F58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="11.1640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -2301,12 +2301,12 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>rD, pS</t>
+          <t>rD</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Port read</t>
+          <t>Port read (UART receive, clears the port IRQ)</t>
         </is>
       </c>
       <c r="E53" s="8" t="n"/>
@@ -2319,66 +2319,50 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>pD, rS</t>
+          <t>rS</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Port write</t>
+          <t>Port write (UART transmit)</t>
         </is>
       </c>
       <c r="E54" s="8" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>PTSR</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>rD</t>
-        </is>
-      </c>
-      <c r="D55" s="9" t="inlineStr">
-        <is>
-          <t>Port state read</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="n"/>
-    </row>
-    <row r="56">
-      <c r="B56" s="10" t="inlineStr">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="C56" s="121" t="n"/>
-      <c r="D56" s="121" t="n"/>
-      <c r="E56" s="121" t="n"/>
-    </row>
-    <row r="57" ht="17" customHeight="1">
-      <c r="B57" s="13" t="inlineStr">
+      <c r="C55" s="121" t="n"/>
+      <c r="D55" s="121" t="n"/>
+      <c r="E55" s="121" t="n"/>
+    </row>
+    <row r="56" ht="17" customHeight="1">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>SVC</t>
         </is>
       </c>
-      <c r="C57" s="14" t="n"/>
-      <c r="D57" s="15" t="inlineStr">
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="15" t="inlineStr">
         <is>
           <t>Supervisor call</t>
         </is>
       </c>
-      <c r="E57" s="14" t="n"/>
-    </row>
+      <c r="E56" s="14" t="n"/>
+    </row>
+    <row r="57"/>
+    <row r="58"/>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B56:E56"/>
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="D2:E3"/>
     <mergeCell ref="B52:E52"/>
     <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B55:E55"/>
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>

</xml_diff>